<commit_message>
Excel-only separation: Remove non-Excel features and update UI
- Move Instructions feature to Experimented/api/
- Move non-Excel UI templates to BACKUP/web/templates/
- Clean up api/routes.py: Keep only health and screenshots routes
- Clean up api/app.py: Remove non-Excel route registrations
- Update index.html: Remove non-Excel UI sections and navigation
- Update UI branding to Excel Test Generator focus
- Backup original api/routes.py to BACKUP/api_routes_original.py
</commit_message>
<xml_diff>
--- a/test_case.xlsx
+++ b/test_case.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10110"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10118"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lollal/Documents/ai-agent-qa/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42B7CAE8-5BA9-F941-A0E4-228898D50982}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8962FFBA-9979-0946-85B8-7616C7B110FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17480" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="68800" windowHeight="26400" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="52">
   <si>
     <t>Step</t>
   </si>
@@ -49,12 +49,12 @@
     <t>Optional</t>
   </si>
   <si>
+    <t>Modal</t>
+  </si>
+  <si>
     <t>https://hub-stage.datacommons.cancer.gov/</t>
   </si>
   <si>
-    <t>N/A</t>
-  </si>
-  <si>
     <t>page</t>
   </si>
   <si>
@@ -76,18 +76,24 @@
     <t>click</t>
   </si>
   <si>
+    <t xml:space="preserve">yes </t>
+  </si>
+  <si>
     <t>(//a[@id='header-navbar-login-button'])[1]</t>
   </si>
   <si>
     <t>link</t>
   </si>
   <si>
+    <t>https://auth.nih.gov/CertAuthV3/forms/nihl/LoginMFA.aspx</t>
+  </si>
+  <si>
+    <t>(//*[normalize-space(.)='Login.gov'])[1]</t>
+  </si>
+  <si>
     <t>https://secure.login.gov</t>
   </si>
   <si>
-    <t>(//*[normalize-space(.)='Login.gov'])[1]</t>
-  </si>
-  <si>
     <t>//input[@type='email']</t>
   </si>
   <si>
@@ -118,7 +124,13 @@
     <t>${TOTP_CODE}</t>
   </si>
   <si>
-    <t>//input[@name='action']</t>
+    <t>https://secure.login.gov/login/two_factor/sms</t>
+  </si>
+  <si>
+    <t>https://ras.nih.gov/auth/oauth/v2/authorize/consent</t>
+  </si>
+  <si>
+    <t>//input[@name='action' and @value='Grant']</t>
   </si>
   <si>
     <t>https://hub-stage.datacommons.cancer.gov/data-submissions</t>
@@ -128,13 +140,49 @@
   </si>
   <si>
     <t>//button[normalize-space(.)='Create a Data Submission']</t>
+  </si>
+  <si>
+    <t>//div[@data-testid="create-data-submission-dialog-data-commons-input"]//div[@id="mui-component-select-dataCommons" and @role="button"]</t>
+  </si>
+  <si>
+    <t>dropdown</t>
+  </si>
+  <si>
+    <t>GC</t>
+  </si>
+  <si>
+    <t>//ul[@role="listbox"]//li[@role="option" and normalize-space(.)="GC"]</t>
+  </si>
+  <si>
+    <t>option</t>
+  </si>
+  <si>
+    <t>//div[@id="mui-component-select-studyID" and @role="button"]</t>
+  </si>
+  <si>
+    <t>//ul[@role="listbox"]//li[@role="option" and normalize-space(.)="NewTestSpn_laxmi"]</t>
+  </si>
+  <si>
+    <t>NewTestSpn_laxmi</t>
+  </si>
+  <si>
+    <t>(//*[@data-testid="create-submission-dialog"])//input[@name='name']</t>
+  </si>
+  <si>
+    <t>TIMESTAMP</t>
+  </si>
+  <si>
+    <t>${TIMESTAMP}</t>
+  </si>
+  <si>
+    <t>(//*[@data-testid="create-submission-dialog"])//button[@data-testid='create-data-submission-dialog-create-button']</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -144,9 +192,13 @@
     </font>
     <font>
       <b/>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <family val="2"/>
+      <sz val="16"/>
+      <name val="Calibri (Body)"/>
+    </font>
+    <font>
+      <sz val="16"/>
+      <color theme="1"/>
+      <name val="Calibri (Body)"/>
     </font>
   </fonts>
   <fills count="2">
@@ -184,11 +236,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -491,16 +544,23 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I16"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:J21"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="21" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="4.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="47.1640625" customWidth="1"/>
-    <col min="3" max="3" width="75.1640625" customWidth="1"/>
-    <col min="4" max="4" width="8.6640625" customWidth="1"/>
+    <col min="1" max="1" width="6.33203125" style="2" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="69.6640625" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="165.83203125" style="2" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.83203125" style="2" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.5" style="2" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14.5" style="2" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="31.1640625" style="2" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="12.83203125" style="2" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="11.1640625" style="2" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="8.5" style="2" bestFit="1" customWidth="1"/>
+    <col min="11" max="16384" width="9" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -528,326 +588,480 @@
       <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A2">
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A2" s="2">
         <v>1</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="I2" s="2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="H3" s="2">
+        <v>3000</v>
+      </c>
+      <c r="I3" s="2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A4" s="2">
+        <v>2</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="I4" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="J4" s="2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A5" s="2">
+        <v>3</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="I5" s="2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A6" s="2">
+        <v>4</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="I6" s="2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A7" s="2">
+        <v>5</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="G7" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="I7" s="2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A8" s="2">
+        <v>6</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="G8" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="I8" s="2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A9" s="2">
+        <v>7</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="I9" s="2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A10" s="2">
+        <v>8</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="G10" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="I10" s="2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A11" s="2">
         <v>9</v>
       </c>
-      <c r="C2" t="s">
+      <c r="B11" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="I11" s="2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A12" s="2">
         <v>10</v>
       </c>
-      <c r="D2" t="s">
+      <c r="B12" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="I12" s="2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A13" s="2">
         <v>11</v>
       </c>
-      <c r="E2" t="s">
+      <c r="B13" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="I13" s="2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A14" s="2">
         <v>12</v>
       </c>
-      <c r="I2" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
+      <c r="B14" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="H14" s="2">
+        <v>3000</v>
+      </c>
+      <c r="I14" s="2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A15" s="2">
         <v>13</v>
       </c>
-      <c r="B3" t="s">
-        <v>9</v>
-      </c>
-      <c r="C3" t="s">
-        <v>10</v>
-      </c>
-      <c r="D3" t="s">
-        <v>11</v>
-      </c>
-      <c r="E3" t="s">
+      <c r="B15" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="E15" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="H15" s="2">
+        <v>3000</v>
+      </c>
+      <c r="I15" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="J15" s="2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A16" s="2">
+        <v>13</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="E16" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="G16" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="H16" s="2">
+        <v>3000</v>
+      </c>
+      <c r="I16" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="J16" s="2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A17" s="2">
         <v>14</v>
       </c>
-      <c r="H3">
+      <c r="B17" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="E17" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="G17" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="H17" s="2">
         <v>3000</v>
       </c>
-      <c r="I3" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A4">
-        <v>2</v>
-      </c>
-      <c r="B4" t="s">
-        <v>9</v>
-      </c>
-      <c r="C4" t="s">
+      <c r="I17" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="J17" s="2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A18" s="2">
         <v>15</v>
       </c>
-      <c r="D4" t="s">
+      <c r="B18" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="E18" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="H18" s="2">
+        <v>3000</v>
+      </c>
+      <c r="I18" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="J18" s="2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A19" s="2">
         <v>16</v>
       </c>
-      <c r="E4" t="s">
-        <v>17</v>
-      </c>
-      <c r="I4" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A5">
-        <v>3</v>
-      </c>
-      <c r="B5" t="s">
-        <v>9</v>
-      </c>
-      <c r="C5" t="s">
+      <c r="B19" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="E19" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="G19" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="H19" s="2">
+        <v>3000</v>
+      </c>
+      <c r="I19" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="J19" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="D5" t="s">
-        <v>19</v>
-      </c>
-      <c r="E5" t="s">
-        <v>17</v>
-      </c>
-      <c r="I5" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A6">
-        <v>4</v>
-      </c>
-      <c r="B6" t="s">
-        <v>20</v>
-      </c>
-      <c r="C6" t="s">
-        <v>21</v>
-      </c>
-      <c r="D6" t="s">
+    </row>
+    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A20" s="2">
+        <v>17</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="E20" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="F20" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="G20" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="H20" s="2">
+        <v>3000</v>
+      </c>
+      <c r="I20" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="J20" s="2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A21" s="2">
+        <v>18</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="D21" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="E6" t="s">
-        <v>17</v>
-      </c>
-      <c r="I6" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A7">
-        <v>5</v>
-      </c>
-      <c r="B7" t="s">
-        <v>20</v>
-      </c>
-      <c r="C7" t="s">
-        <v>22</v>
-      </c>
-      <c r="D7" t="s">
-        <v>23</v>
-      </c>
-      <c r="E7" t="s">
-        <v>24</v>
-      </c>
-      <c r="G7" t="s">
-        <v>25</v>
-      </c>
-      <c r="I7" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A8">
-        <v>6</v>
-      </c>
-      <c r="B8" t="s">
-        <v>20</v>
-      </c>
-      <c r="C8" t="s">
-        <v>26</v>
-      </c>
-      <c r="D8" t="s">
-        <v>23</v>
-      </c>
-      <c r="E8" t="s">
-        <v>24</v>
-      </c>
-      <c r="G8" t="s">
-        <v>27</v>
-      </c>
-      <c r="I8" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A9">
-        <v>7</v>
-      </c>
-      <c r="B9" t="s">
-        <v>20</v>
-      </c>
-      <c r="C9" t="s">
-        <v>28</v>
-      </c>
-      <c r="D9" t="s">
-        <v>16</v>
-      </c>
-      <c r="E9" t="s">
-        <v>17</v>
-      </c>
-      <c r="I9" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A10">
-        <v>8</v>
-      </c>
-      <c r="B10" t="s">
-        <v>20</v>
-      </c>
-      <c r="C10" t="s">
-        <v>29</v>
-      </c>
-      <c r="D10" t="s">
-        <v>23</v>
-      </c>
-      <c r="E10" t="s">
-        <v>24</v>
-      </c>
-      <c r="F10" t="s">
-        <v>30</v>
-      </c>
-      <c r="G10" t="s">
-        <v>31</v>
-      </c>
-      <c r="I10" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A11">
-        <v>9</v>
-      </c>
-      <c r="B11" t="s">
-        <v>20</v>
-      </c>
-      <c r="C11" t="s">
-        <v>10</v>
-      </c>
-      <c r="D11" t="s">
-        <v>11</v>
-      </c>
-      <c r="E11" t="s">
-        <v>14</v>
-      </c>
-      <c r="H11">
-        <v>5000</v>
-      </c>
-      <c r="I11" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A12">
-        <v>10</v>
-      </c>
-      <c r="B12" t="s">
-        <v>20</v>
-      </c>
-      <c r="C12" t="s">
-        <v>28</v>
-      </c>
-      <c r="D12" t="s">
-        <v>16</v>
-      </c>
-      <c r="E12" t="s">
-        <v>17</v>
-      </c>
-      <c r="I12" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A13">
-        <v>11</v>
-      </c>
-      <c r="B13" t="s">
-        <v>20</v>
-      </c>
-      <c r="C13" t="s">
-        <v>10</v>
-      </c>
-      <c r="D13" t="s">
-        <v>11</v>
-      </c>
-      <c r="E13" t="s">
-        <v>14</v>
-      </c>
-      <c r="H13">
-        <v>2000</v>
-      </c>
-      <c r="I13" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A14">
-        <v>12</v>
-      </c>
-      <c r="B14" t="s">
-        <v>20</v>
-      </c>
-      <c r="C14" t="s">
-        <v>32</v>
-      </c>
-      <c r="D14" t="s">
-        <v>16</v>
-      </c>
-      <c r="E14" t="s">
-        <v>17</v>
-      </c>
-      <c r="I14" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A15">
-        <v>14</v>
-      </c>
-      <c r="B15" t="s">
-        <v>33</v>
-      </c>
-      <c r="C15" t="s">
-        <v>34</v>
-      </c>
-      <c r="D15" t="s">
-        <v>16</v>
-      </c>
-      <c r="E15" t="s">
-        <v>17</v>
-      </c>
-      <c r="I15" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A16">
-        <v>15</v>
-      </c>
-      <c r="B16" t="s">
-        <v>33</v>
-      </c>
-      <c r="C16" t="s">
-        <v>35</v>
-      </c>
-      <c r="D16" t="s">
-        <v>16</v>
-      </c>
-      <c r="E16" t="s">
-        <v>17</v>
-      </c>
-      <c r="I16" t="b">
-        <v>0</v>
+      <c r="E21" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="H21" s="2">
+        <v>3000</v>
+      </c>
+      <c r="I21" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="J21" s="2" t="s">
+        <v>18</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix modal XPaths: Add create-submission-dialog scoping to steps 16-19
- Step 16: Data Commons dropdown - now modal-scoped
- Step 16b: GC option - now modal-scoped
- Step 17: Study ID dropdown - now modal-scoped
- Step 17b: NewTestSpn_laxmi option - now modal-scoped

All XPaths now include: (//*[@data-testid="create-submission-dialog"]) prefix
</commit_message>
<xml_diff>
--- a/test_case.xlsx
+++ b/test_case.xlsx
@@ -938,6 +938,11 @@
           <t>click</t>
         </is>
       </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>(//*[@data-testid="create-submission-dialog"])//div[@id="mui-component-select-dataCommons" and @role="button"]</t>
+        </is>
+      </c>
       <c r="I17" t="b">
         <v>0</v>
       </c>
@@ -966,6 +971,11 @@
       <c r="E18" t="inlineStr">
         <is>
           <t>click</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>(//*[@data-testid="create-submission-dialog"])//ul[@role="listbox"]//li[@role="option" and normalize-space(.)="GC"]</t>
         </is>
       </c>
       <c r="I18" t="b">
@@ -996,6 +1006,11 @@
           <t>click</t>
         </is>
       </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>(//*[@data-testid="create-submission-dialog"])//div[@id="mui-component-select-studyID" and @role="button"]</t>
+        </is>
+      </c>
       <c r="I19" t="b">
         <v>0</v>
       </c>
@@ -1024,6 +1039,11 @@
       <c r="E20" t="inlineStr">
         <is>
           <t>click</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>(//*[@data-testid="create-submission-dialog"])//ul[@role="listbox"]//li[@role="option" and normalize-space(.)="NewTestSpn_laxmi"]</t>
         </is>
       </c>
       <c r="I20" t="b">

</xml_diff>

<commit_message>
Add missing steps 18-19: Submission Name input and Create button
- Step 18: Fill Submission Name input with 'Timestamp' value
- Step 19: Click Create button in modal dialog
- Both steps include modal-scoped XPaths with create-submission-dialog context
</commit_message>
<xml_diff>
--- a/test_case.xlsx
+++ b/test_case.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I20"/>
+  <dimension ref="A1:I22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1050,6 +1050,77 @@
         <v>0</v>
       </c>
     </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>18</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>https://hub-stage.datacommons.cancer.gov/data-submissions</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>//input[@name='name']</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>input</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>fill</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>(//*[@data-testid="create-submission-dialog"])//input[@name='name']</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>Timestamp</t>
+        </is>
+      </c>
+      <c r="I21" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>19</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>https://hub-stage.datacommons.cancer.gov/data-submissions</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>//button[@data-testid='create-data-submission-dialog-create-button']</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>button</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>click</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>(//*[@data-testid="create-submission-dialog"])//button[@data-testid='create-data-submission-dialog-create-button']</t>
+        </is>
+      </c>
+      <c r="I22" t="b">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>